<commit_message>
Updated on 12-11-2023 at 19:49
</commit_message>
<xml_diff>
--- a/output/solution_cubic.xlsx
+++ b/output/solution_cubic.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,25 +444,49 @@
       <c r="F1" s="1" t="n">
         <v>4</v>
       </c>
+      <c r="G1" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.969143</v>
+        <v>2.133</v>
       </c>
       <c r="C2" t="n">
-        <v>1.033761</v>
+        <v>-1.929</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1007038</v>
+        <v>-1.586</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1061653</v>
+        <v>0.791</v>
       </c>
       <c r="F2" t="n">
-        <v>2.148787</v>
+        <v>121.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>108</v>
+      </c>
+      <c r="H2" t="n">
+        <v>39886</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2754</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.052</v>
       </c>
     </row>
     <row r="3">
@@ -470,19 +494,31 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.988122</v>
+        <v>2.443</v>
       </c>
       <c r="C3" t="n">
-        <v>1.01935</v>
+        <v>-3.276</v>
       </c>
       <c r="D3" t="n">
-        <v>0.09763946</v>
+        <v>-0.55</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.104015</v>
+        <v>0.608</v>
       </c>
       <c r="F3" t="n">
-        <v>1.701151</v>
+        <v>75.20999999999999</v>
+      </c>
+      <c r="G3" t="n">
+        <v>173</v>
+      </c>
+      <c r="H3" t="n">
+        <v>60064</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4109</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="4">
@@ -490,19 +526,31 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.995534</v>
+        <v>2.371</v>
       </c>
       <c r="C4" t="n">
-        <v>1.035261</v>
+        <v>-2.89</v>
       </c>
       <c r="D4" t="n">
-        <v>0.09806779</v>
+        <v>-0.918</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1059407</v>
+        <v>0.695</v>
       </c>
       <c r="F4" t="n">
-        <v>1.328797</v>
+        <v>52.55</v>
+      </c>
+      <c r="G4" t="n">
+        <v>148</v>
+      </c>
+      <c r="H4" t="n">
+        <v>47297</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3300</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.067</v>
       </c>
     </row>
     <row r="5">
@@ -510,19 +558,31 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2.012014</v>
+        <v>2.073</v>
       </c>
       <c r="C5" t="n">
-        <v>1.031959</v>
+        <v>-1.737</v>
       </c>
       <c r="D5" t="n">
-        <v>0.09510908</v>
+        <v>-1.516</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1054367</v>
+        <v>0.778</v>
       </c>
       <c r="F5" t="n">
-        <v>1.073974</v>
+        <v>31.62</v>
+      </c>
+      <c r="G5" t="n">
+        <v>196</v>
+      </c>
+      <c r="H5" t="n">
+        <v>61655</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4413</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -530,19 +590,31 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2.018474</v>
+        <v>2.014</v>
       </c>
       <c r="C6" t="n">
-        <v>1.01888</v>
+        <v>-0.612</v>
       </c>
       <c r="D6" t="n">
-        <v>0.09534891</v>
+        <v>-2.266</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1038468</v>
+        <v>0.9</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8361448</v>
+        <v>10.8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>163</v>
+      </c>
+      <c r="H6" t="n">
+        <v>45680</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3198</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.068</v>
       </c>
     </row>
     <row r="7">
@@ -550,19 +622,31 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>2.018972</v>
+        <v>1.002</v>
       </c>
       <c r="C7" t="n">
-        <v>1.012884</v>
+        <v>0.996</v>
       </c>
       <c r="D7" t="n">
-        <v>0.09749349</v>
+        <v>-2.998</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1037276</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6123674</v>
+        <v>0.0006061</v>
+      </c>
+      <c r="G7" t="n">
+        <v>198</v>
+      </c>
+      <c r="H7" t="n">
+        <v>62852</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4225</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.103</v>
       </c>
     </row>
     <row r="8">
@@ -570,19 +654,31 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>2.01917</v>
+        <v>1.005</v>
       </c>
       <c r="C8" t="n">
-        <v>1.018431</v>
+        <v>0.991</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09954157</v>
+        <v>-2.995</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.1038304</v>
+        <v>0.999</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4168652</v>
+        <v>0.00056</v>
+      </c>
+      <c r="G8" t="n">
+        <v>231</v>
+      </c>
+      <c r="H8" t="n">
+        <v>76275</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5230</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.123</v>
       </c>
     </row>
     <row r="9">
@@ -590,19 +686,31 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>2.005971</v>
+        <v>1.009</v>
       </c>
       <c r="C9" t="n">
-        <v>1.01312</v>
+        <v>0.985</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1018362</v>
+        <v>-2.993</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1030356</v>
+        <v>0.999</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2497143</v>
+        <v>0.0004961</v>
+      </c>
+      <c r="G9" t="n">
+        <v>295</v>
+      </c>
+      <c r="H9" t="n">
+        <v>90799</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6160</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.145</v>
       </c>
     </row>
     <row r="10">
@@ -610,19 +718,31 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.994068</v>
+        <v>1.009</v>
       </c>
       <c r="C10" t="n">
-        <v>1.006989</v>
+        <v>0.982</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1038632</v>
+        <v>-2.991</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.102122</v>
+        <v>0.999</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1144112</v>
+        <v>0.0004434</v>
+      </c>
+      <c r="G10" t="n">
+        <v>384</v>
+      </c>
+      <c r="H10" t="n">
+        <v>126062</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8372</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.203</v>
       </c>
     </row>
     <row r="11">
@@ -630,19 +750,31 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>2.000078</v>
+        <v>1.01</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9991906</v>
+        <v>0.98</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1001741</v>
+        <v>-2.991</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.09981659</v>
+        <v>0.999</v>
       </c>
       <c r="F11" t="n">
-        <v>0.001147395</v>
+        <v>0.0003869</v>
+      </c>
+      <c r="G11" t="n">
+        <v>529</v>
+      </c>
+      <c r="H11" t="n">
+        <v>163881</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11070</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.257</v>
       </c>
     </row>
     <row r="12">
@@ -650,119 +782,31 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>2.000284</v>
+        <v>1.013</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9988813</v>
+        <v>0.977</v>
       </c>
       <c r="D12" t="n">
-        <v>0.100059</v>
+        <v>-2.989</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0997348</v>
+        <v>0.999</v>
       </c>
       <c r="F12" t="n">
-        <v>0.001084392</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="n">
-        <v>2.000385</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.9988026</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.09997955</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-0.09969793</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.001029498</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="n">
-        <v>2.000481</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.9987492</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.09989764</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-0.09966404</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.0009720265</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="n">
-        <v>2.000635</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.9986155</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.09979018000000001</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-0.09961100000000001</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.0009155347</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="n">
-        <v>2.000552</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.9987844</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.09977503</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-0.09962686</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.0008693338</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="n">
-        <v>2.000505</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.9986042000000001</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.09975684</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-0.09960478</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.0008263589</v>
+        <v>0.0003481</v>
+      </c>
+      <c r="G12" t="n">
+        <v>613</v>
+      </c>
+      <c r="H12" t="n">
+        <v>193966</v>
+      </c>
+      <c r="I12" t="n">
+        <v>13328</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>